<commit_message>
Atualiza README.md com fontes de notícias e adiciona novos dados ao CSV e ao log de coleta
</commit_message>
<xml_diff>
--- a/data/relatorio_sentimentos.xlsx
+++ b/data/relatorio_sentimentos.xlsx
@@ -511,42 +511,42 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
         <v>2</v>
       </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.792</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
         <v>1</v>
       </c>
-      <c r="E2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.8882</v>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>NEUTRO</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>28.6</v>
-      </c>
-      <c r="J2" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="K2" t="n">
-        <v>3</v>
-      </c>
       <c r="L2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M2" t="n">
-        <v>14.3</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -560,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1174,6 +1174,231 @@
         </is>
       </c>
       <c r="Q8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-24T15:47:36</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BBDC4</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>cac3406bcbd4</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Bradesco abre 225 vagas de emprego no Brasil com oportunidades em tecnologia, negócios e segurança da informação</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Bradesco abre 225 vagas de emprego no Brasil com oportunidades em tecnologia, negócios e segurança da informação&amp;nbsp;&amp;nbsp;JC Concursos</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi9AFBVV95cUxOZTNvejdEODhSOEZiQkxfUTNoQjZQcXZRVlB3UmhvcUJKazlCNk5keUJRSEJGOUI0amhXYjZKaGRpYlFpTHkzVFdkc3hJMFlqelVOQXpLSGZzQ3dIMFpmWTNra2wxYU4yN2Itbmp1SGQxakpnR3RWakZoQzNOLVNTVlMxRnotdUY4eDk2Wk41VkdORUY0azVzUzNfY0ZReF9oM3MwOGc5QnZkUFhZNmx1NVRJbDhaMzVKVDJvMnA4OXh6TnBORFVHM2pRSHo3ZUtlTS03N0QybS1LN0tyQzhudndQR203RU1RdGlwN3VlTE1EeHBq0gH6AUFVX3lxTFBvTHlyWVdybTAwaVloXzlnb2syV3A1M0lTeDd6S3NncmxBeVdRS1Q1RENpRURES1RJemtGdl9iMUxkNlFhM3JkczZLZVhiYi11VXdtbUN6QmxmWFFhMkgzcUdqN3lzbndXX1A5OVdGU21LQmdSb1ZUMUxrZjdiMktTMEFBdVo4VnFGbmY1SHZ3UGxlVkZjZE1qUkxpMUQ1ek9OT2F5NVQxRWNDUU5LUXFfMmpYdjgyb3AxdUs1NENhVHRwWF81aFlXLVNRWWtuSGNOdTZKN1VRRE1CQ1VCRzVDNzNzYVZDWHZlZ2JSUFRCQUJPZFlsaGpUNGc?oc=5</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>JC Concursos</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-05-22T21:36:00+00:00</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Bradesco</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>POSITIVO</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>0.841</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Bradesco opens 225 job vacancies in Brazil with opportunities in technology, business and information security. Bradesco opens 225 job vacancies in Brazil with opportunities in technology, business and information security&amp;nbsp;&amp;nbsp;JC Concursos</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-24T15:47:36</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BBDC4</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>d83715720261</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Bradesco oferece mais de 80 cursos gratuitos com certificado online</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Bradesco oferece mais de 80 cursos gratuitos com certificado online&amp;nbsp;&amp;nbsp;Serra Noticiário</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxQaFRzVENxeS1RbGx3WDBHZEFtZkJ5NC1KTi13aHc5X25uMGVaLXZ6ekNVUzAwcDBBaDBUblQzN0ptSXZ2U284RzNKTGRPVFczY2VDYUIyX0hUOGpNZTVNYnNjOFZnc0E5ZndjVG5UYnhkV1V2d0dJWmw2bkNSaHhNYjMyM3NPRlFiUkNfbXNoQ0tYVW5laV9hYzhIc2dTb2Fx?oc=5</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Serra Noticiário</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-05-23T18:25:00+00:00</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Bradesco</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>0.9221</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Bradesco offers more than 80 free courses with online certificates. Bradesco offers more than 80 free courses with online certificate&amp;nbsp;&amp;nbsp;Serra Noticiário</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-24T15:47:36</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BBDC4</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>9ae5cbab2aa4</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Bradesco Seguros divulga ações durante Maio Amarelo</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Bradesco Seguros divulga ações durante Maio Amarelo&amp;nbsp;&amp;nbsp;Grandes Nomes da Propaganda</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxPT0ZBekUwdzJoUG9uc3E3Wk4tZ1MtUGFSS0dHc09KYXZrc012SzRNZlprWGl1RF9kUW0ya0lDV1hJbzdWYldsb3pVTU9DMHVmSmhSQURkTzBLd3lhV0VhSGdTLXpfVENmQUtmWkNvYWxfMGozOXdQbDIwUmxRMXFtbkpfbHRNTGxiQ1d0Si1ZbEN5cTBWRmk4ek9nSWQxQVRBbHZPUW5aekd1WkpU?oc=5</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Grandes Nomes da Propaganda</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-05-23T05:01:00+00:00</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Bradesco</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>0.613</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Bradesco Seguros publishes actions during Yellow May. Bradesco Seguros announces actions during Yellow May&amp;nbsp;&amp;nbsp;Big Names in Advertising</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1221,10 +1446,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>